<commit_message>
Mängdavtagning: mängdslag Form (m²), Längd (m) och Armering (kg) – egen egenskap, enhetskontroll mot objektens mått och egen koppling till poster per slag
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECqjXEGHxiKAfdmAab72Dz
</commit_message>
<xml_diff>
--- a/test/fixtures/mf_test.xlsx
+++ b/test/fixtures/mf_test.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -852,6 +852,113 @@
         <v>14498</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ESB.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Formar av valfri typ | h &gt; 250 | grundsulor</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>542</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1499</v>
+      </c>
+      <c r="O10" t="n">
+        <v>750</v>
+      </c>
+      <c r="P10" t="n">
+        <v>432</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>153</v>
+      </c>
+      <c r="S10" t="n">
+        <v>16</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3392</v>
+      </c>
+      <c r="V10" t="n">
+        <v>542</v>
+      </c>
+      <c r="W10" t="n">
+        <v>1499</v>
+      </c>
+      <c r="X10" t="n">
+        <v>750</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>432</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>153</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>16</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>3392</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>väggar</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>5846</v>
+      </c>
+      <c r="O11" t="n">
+        <v>6946</v>
+      </c>
+      <c r="P11" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>63</v>
+      </c>
+      <c r="R11" t="n">
+        <v>149</v>
+      </c>
+      <c r="T11" t="n">
+        <v>13074</v>
+      </c>
+      <c r="W11" t="n">
+        <v>5846</v>
+      </c>
+      <c r="X11" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>70</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>63</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>149</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>13128</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>